<commit_message>
docs: add the offer-category accordion check to the UAT checklist
- TESTING-GUIDE.md: a Resident bullet — the "Notify me about" list is a
  tap-to-expand accordion (~6 collapsed groups, chevron rotate, count badge,
  multi-open); flagged to check on the installed APK.
- Single-Point-Test-Cases.xlsx: new case M9-10 in the M9 sheet + Summary count.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Single-Point-Test-Cases.xlsx
+++ b/docs/Single-Point-Test-Cases.xlsx
@@ -523,6 +523,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -672,7 +673,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
@@ -817,7 +818,7 @@
         </is>
       </c>
       <c r="C24" s="3" t="n">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>
@@ -831,7 +832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1431,6 +1432,64 @@
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>M9-10</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Notifications &amp; in-app inbox</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Offer category picker</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Category list is a tap-to-expand accordion (mobile)</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Resident signed in on the installed Android APK; Settings &gt; Offer notifications</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>1. Open Settings &gt; Offer notifications &gt; 'Notify me about'  2. Tap a group header (e.g. Home &amp; Maintenance)  3. Toggle a sub-category on  4. Collapse the group  5. Expand a second group</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>The list shows ~6 collapsed group rows (not a long toggle scroll); a tap expands the group's sub-toggles and rotates the chevron; a collapsed group with a selection shows a count badge; more than one group can be open at once; expand/collapse eases (native animation).</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>

</xml_diff>